<commit_message>
Enforce unique article numbers; inline error + clear on edit/ZurÃ¼ck
- Backend: reject duplicate full_article_number on BOM generation

- Inline duplicate warning in Neue Konfiguration card; clear on input and on ZurÃ¼ck

- ZurÃ¼ck from BOM output deletes temp config so same article can be reused

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/main excel/main.xlsx
+++ b/main excel/main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\05 Entwicklung\01 Projekte\In Progress\Stücklistenkonfigurator\Ausführungsdateien\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1454F275-CB51-4F9E-AB0D-2F6E0D524C94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59235005-5EC8-4825-9B63-1B91BF80BE5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Schacht" sheetId="1" r:id="rId1"/>
@@ -190,7 +190,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="254">
   <si>
     <t>Artikelnummer</t>
   </si>
@@ -919,6 +919,39 @@
   </si>
   <si>
     <t>GN 2 | GN X1 | GN X2 | GN X3 | GN X4</t>
+  </si>
+  <si>
+    <t>Stumpfschweiß-Reduktion DA 160 / 125 kurz</t>
+  </si>
+  <si>
+    <t>Stumpfschweiß-Reduktion DA 200 / 125 kurz</t>
+  </si>
+  <si>
+    <t>Stumpfschweiß-Reduktion DA 200 / 180 kurz</t>
+  </si>
+  <si>
+    <t>Stumpfschweiß-Reduktion DA 225 / 110 kurz</t>
+  </si>
+  <si>
+    <t>Stumpfschweiß-Reduktion DA 225 / 140 kurz</t>
+  </si>
+  <si>
+    <t>Stumpfschweiß-Reduktion DA 225 / 160 kurz</t>
+  </si>
+  <si>
+    <t>Stumpfschweiß-Reduktion DA 225 / 180 kurz</t>
+  </si>
+  <si>
+    <t>Stumpfschweiß-Reduktion DA 225 / 200 kurz</t>
+  </si>
+  <si>
+    <t>Stumpfschweiß-Reduktion DA 250 / 160 kurz</t>
+  </si>
+  <si>
+    <t>Stumpfschweiß-Reduktion DA 250 / 200 kurz</t>
+  </si>
+  <si>
+    <t>Stumpfschweiß-Reduktion DA 250 / 225 kurz</t>
   </si>
 </sst>
 </file>
@@ -1136,15 +1169,15 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1924,16 +1957,16 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="33" t="s">
         <v>182</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="22" t="s">
@@ -2426,16 +2459,16 @@
       <c r="H35" s="5"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="30" t="s">
+      <c r="A36" s="33" t="s">
         <v>183</v>
       </c>
-      <c r="B36" s="31"/>
-      <c r="C36" s="31"/>
-      <c r="D36" s="31"/>
-      <c r="E36" s="31"/>
-      <c r="F36" s="31"/>
-      <c r="G36" s="31"/>
-      <c r="H36" s="31"/>
+      <c r="B36" s="34"/>
+      <c r="C36" s="34"/>
+      <c r="D36" s="34"/>
+      <c r="E36" s="34"/>
+      <c r="F36" s="34"/>
+      <c r="G36" s="34"/>
+      <c r="H36" s="34"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="22" t="s">
@@ -5449,7 +5482,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr codeName="Tabelle1"/>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="15" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
@@ -5754,19 +5787,19 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="32">
+      <c r="A18" s="30">
         <v>140</v>
       </c>
-      <c r="B18" s="33">
+      <c r="B18" s="31">
         <v>75</v>
       </c>
-      <c r="C18" s="32">
+      <c r="C18" s="30">
         <v>2002052</v>
       </c>
-      <c r="D18" s="33" t="s">
+      <c r="D18" s="31" t="s">
         <v>236</v>
       </c>
-      <c r="E18" s="34">
+      <c r="E18" s="32">
         <v>2</v>
       </c>
     </row>
@@ -5788,19 +5821,19 @@
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="32">
+      <c r="A20" s="30">
         <v>140</v>
       </c>
-      <c r="B20" s="33">
+      <c r="B20" s="31">
         <v>110</v>
       </c>
-      <c r="C20" s="32">
+      <c r="C20" s="30">
         <v>2000587</v>
       </c>
-      <c r="D20" s="33" t="s">
+      <c r="D20" s="31" t="s">
         <v>237</v>
       </c>
-      <c r="E20" s="34">
+      <c r="E20" s="32">
         <v>2</v>
       </c>
     </row>
@@ -5821,54 +5854,54 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="32" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="32">
+    <row r="22" spans="1:5" s="30" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="30">
         <v>160</v>
       </c>
-      <c r="B22" s="33">
+      <c r="B22" s="31">
         <v>90</v>
       </c>
-      <c r="C22" s="32">
+      <c r="C22" s="30">
         <v>2000599</v>
       </c>
-      <c r="D22" s="33" t="s">
+      <c r="D22" s="31" t="s">
         <v>238</v>
       </c>
-      <c r="E22" s="32">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" s="32" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="32">
+      <c r="E22" s="30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" s="30" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23">
         <v>160</v>
       </c>
-      <c r="B23" s="33">
+      <c r="B23" s="8">
+        <v>110</v>
+      </c>
+      <c r="C23">
+        <v>2000593</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="E23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" s="30" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="30">
+        <v>160</v>
+      </c>
+      <c r="B24" s="31">
         <v>125</v>
       </c>
-      <c r="C23" s="32">
+      <c r="C24" s="30">
         <v>2000595</v>
       </c>
-      <c r="D23" s="33" t="s">
-        <v>109</v>
-      </c>
-      <c r="E23" s="32">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>160</v>
-      </c>
-      <c r="B24" s="8">
-        <v>110</v>
-      </c>
-      <c r="C24">
-        <v>2000593</v>
-      </c>
-      <c r="D24" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="E24">
+      <c r="D24" s="31" t="s">
+        <v>243</v>
+      </c>
+      <c r="E24" s="30">
         <v>2</v>
       </c>
     </row>
@@ -5975,19 +6008,19 @@
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="32">
+      <c r="A31" s="30">
         <v>200</v>
       </c>
-      <c r="B31" s="33">
+      <c r="B31" s="31">
         <v>125</v>
       </c>
-      <c r="C31" s="32">
+      <c r="C31" s="30">
         <v>2000608</v>
       </c>
-      <c r="D31" s="33" t="s">
-        <v>115</v>
-      </c>
-      <c r="E31" s="32">
+      <c r="D31" s="31" t="s">
+        <v>244</v>
+      </c>
+      <c r="E31" s="30">
         <v>2</v>
       </c>
     </row>
@@ -6026,121 +6059,121 @@
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="32">
+      <c r="A34" s="30">
         <v>200</v>
       </c>
-      <c r="B34" s="33">
+      <c r="B34" s="31">
         <v>180</v>
       </c>
-      <c r="C34" s="32">
+      <c r="C34" s="30">
         <v>2000610</v>
       </c>
-      <c r="D34" s="33" t="s">
-        <v>116</v>
-      </c>
-      <c r="E34" s="32">
+      <c r="D34" s="31" t="s">
+        <v>245</v>
+      </c>
+      <c r="E34" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="32">
+      <c r="A35" s="30">
         <v>225</v>
       </c>
-      <c r="B35" s="33">
+      <c r="B35" s="31">
         <v>110</v>
       </c>
-      <c r="C35" s="32">
+      <c r="C35" s="30">
         <v>2002054</v>
       </c>
-      <c r="D35" s="33" t="s">
-        <v>116</v>
-      </c>
-      <c r="E35" s="32">
+      <c r="D35" s="31" t="s">
+        <v>246</v>
+      </c>
+      <c r="E35" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="32">
+      <c r="A36" s="30">
         <v>225</v>
       </c>
-      <c r="B36" s="33">
+      <c r="B36" s="31">
         <v>140</v>
       </c>
-      <c r="C36" s="32">
+      <c r="C36" s="30">
         <v>2002055</v>
       </c>
-      <c r="D36" s="33" t="s">
-        <v>116</v>
-      </c>
-      <c r="E36" s="32">
+      <c r="D36" s="31" t="s">
+        <v>247</v>
+      </c>
+      <c r="E36" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="32">
+      <c r="A37" s="30">
         <v>225</v>
       </c>
-      <c r="B37" s="33">
+      <c r="B37" s="31">
         <v>160</v>
       </c>
-      <c r="C37" s="32">
+      <c r="C37" s="30">
         <v>2001702</v>
       </c>
-      <c r="D37" s="33" t="s">
-        <v>116</v>
-      </c>
-      <c r="E37" s="32">
+      <c r="D37" s="31" t="s">
+        <v>248</v>
+      </c>
+      <c r="E37" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="32">
+      <c r="A38" s="30">
         <v>225</v>
       </c>
-      <c r="B38" s="33">
+      <c r="B38" s="31">
         <v>180</v>
       </c>
-      <c r="C38" s="32">
+      <c r="C38" s="30">
         <v>2002056</v>
       </c>
-      <c r="D38" s="33" t="s">
-        <v>116</v>
-      </c>
-      <c r="E38" s="32">
+      <c r="D38" s="31" t="s">
+        <v>249</v>
+      </c>
+      <c r="E38" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="32">
+      <c r="A39" s="30">
         <v>225</v>
       </c>
-      <c r="B39" s="33">
+      <c r="B39" s="31">
         <v>200</v>
       </c>
-      <c r="C39" s="32">
+      <c r="C39" s="30">
         <v>2002060</v>
       </c>
-      <c r="D39" s="33" t="s">
-        <v>116</v>
-      </c>
-      <c r="E39" s="32">
+      <c r="D39" s="31" t="s">
+        <v>250</v>
+      </c>
+      <c r="E39" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="32">
+      <c r="A40" s="30">
         <v>250</v>
       </c>
-      <c r="B40" s="33">
+      <c r="B40" s="31">
         <v>160</v>
       </c>
-      <c r="C40" s="32">
+      <c r="C40" s="30">
         <v>2001273</v>
       </c>
-      <c r="D40" s="33" t="s">
-        <v>116</v>
-      </c>
-      <c r="E40" s="32">
+      <c r="D40" s="31" t="s">
+        <v>251</v>
+      </c>
+      <c r="E40" s="30">
         <v>2</v>
       </c>
     </row>
@@ -6162,41 +6195,42 @@
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="32">
+      <c r="A42" s="30">
         <v>250</v>
       </c>
-      <c r="B42" s="33">
+      <c r="B42" s="31">
         <v>200</v>
       </c>
-      <c r="C42" s="32">
+      <c r="C42" s="30">
         <v>2000616</v>
       </c>
-      <c r="D42" s="33" t="s">
-        <v>116</v>
-      </c>
-      <c r="E42" s="32">
+      <c r="D42" s="31" t="s">
+        <v>252</v>
+      </c>
+      <c r="E42" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="32">
+      <c r="A43" s="30">
         <v>250</v>
       </c>
-      <c r="B43" s="33">
+      <c r="B43" s="31">
         <v>225</v>
       </c>
-      <c r="C43" s="32">
+      <c r="C43" s="30">
         <v>2002058</v>
       </c>
-      <c r="D43" s="33" t="s">
-        <v>116</v>
-      </c>
-      <c r="E43" s="32">
+      <c r="D43" s="31" t="s">
+        <v>253</v>
+      </c>
+      <c r="E43" s="30">
         <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25"/>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>